<commit_message>
feat: permitir reposicion masiva de stock por SKU
</commit_message>
<xml_diff>
--- a/public/plantilla-productos-hachiko.xlsx
+++ b/public/plantilla-productos-hachiko.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="R52dd550308274324"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV" sheetId="2" r:id="R4ecfa4865a2f4f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="3" r:id="R95611598f3a34700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="R9ebb7379743c45f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSV" sheetId="2" r:id="R43b66d134ae44321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="3" r:id="R1ebb7ee5343b464c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -348,6 +348,7 @@
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="26" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -365,6 +366,7 @@
       <x:c r="L1" s="2"/>
       <x:c r="M1" s="2"/>
       <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
@@ -383,6 +385,7 @@
       <x:c r="L2" s="2"/>
       <x:c r="M2" s="2"/>
       <x:c r="N2" s="2"/>
+      <x:c r="O2" s="2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
@@ -403,10 +406,11 @@
       <x:c r="L3" s="2"/>
       <x:c r="M3" s="2"/>
       <x:c r="N3" s="2"/>
+      <x:c r="O3" s="2"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
-        <x:v>1. Completa las celdas amarillas. SKU y URL se calculan a la derecha (M y N).</x:v>
+        <x:v>1. Producto nuevo: completa sus datos. Reposición: escribe SKU existente (O) y cantidad en Stock (E).</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -421,6 +425,7 @@
       <x:c r="L4" s="2"/>
       <x:c r="M4" s="2"/>
       <x:c r="N4" s="2"/>
+      <x:c r="O4" s="2"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
@@ -439,6 +444,7 @@
       <x:c r="L5" s="2"/>
       <x:c r="M5" s="2"/>
       <x:c r="N5" s="2"/>
+      <x:c r="O5" s="2"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
@@ -457,6 +463,7 @@
       <x:c r="L6" s="2"/>
       <x:c r="M6" s="2"/>
       <x:c r="N6" s="2"/>
+      <x:c r="O6" s="2"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -472,7 +479,7 @@
         <x:v>Precio (CLP) *</x:v>
       </x:c>
       <x:c r="E7" s="8" t="str">
-        <x:v>Stock (un.) *</x:v>
+        <x:v>Stock / sumar *</x:v>
       </x:c>
       <x:c r="F7" s="8" t="str">
         <x:v>Peso (g) *</x:v>
@@ -500,6 +507,9 @@
       </x:c>
       <x:c r="N7" s="8" t="str">
         <x:v>URL automática</x:v>
+      </x:c>
+      <x:c r="O7" s="8" t="str">
+        <x:v>SKU existente (reposición)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -507,7 +517,7 @@
       <x:c r="B8" s="11"/>
       <x:c r="C8" s="9"/>
       <x:c r="D8" s="12"/>
-      <x:c r="E8" s="12"/>
+      <x:c r="E8" s="12" t="str"/>
       <x:c r="F8" s="12"/>
       <x:c r="G8" s="12"/>
       <x:c r="H8" s="12"/>
@@ -516,11 +526,12 @@
       <x:c r="K8" s="9"/>
       <x:c r="L8" s="9"/>
       <x:c r="M8" s="10" t="str">
-        <x:f>IF(A8="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O8&lt;&gt;"",O8,IF(A8="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N8" s="10" t="str">
         <x:f>IF(M8="","",LOWER(M8))</x:f>
       </x:c>
+      <x:c r="O8" s="4" t="str"/>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="11"/>
@@ -536,11 +547,12 @@
       <x:c r="K9" s="9"/>
       <x:c r="L9" s="9"/>
       <x:c r="M9" s="10" t="str">
-        <x:f>IF(A9="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O9&lt;&gt;"",O9,IF(A9="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N9" s="10" t="str">
         <x:f>IF(M9="","",LOWER(M9))</x:f>
       </x:c>
+      <x:c r="O9" s="4"/>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="11"/>
@@ -556,11 +568,12 @@
       <x:c r="K10" s="9"/>
       <x:c r="L10" s="9"/>
       <x:c r="M10" s="10" t="str">
-        <x:f>IF(A10="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O10&lt;&gt;"",O10,IF(A10="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N10" s="10" t="str">
         <x:f>IF(M10="","",LOWER(M10))</x:f>
       </x:c>
+      <x:c r="O10" s="4"/>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="11"/>
@@ -576,11 +589,12 @@
       <x:c r="K11" s="9"/>
       <x:c r="L11" s="9"/>
       <x:c r="M11" s="10" t="str">
-        <x:f>IF(A11="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O11&lt;&gt;"",O11,IF(A11="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N11" s="10" t="str">
         <x:f>IF(M11="","",LOWER(M11))</x:f>
       </x:c>
+      <x:c r="O11" s="4"/>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="11"/>
@@ -596,11 +610,12 @@
       <x:c r="K12" s="9"/>
       <x:c r="L12" s="9"/>
       <x:c r="M12" s="10" t="str">
-        <x:f>IF(A12="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O12&lt;&gt;"",O12,IF(A12="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N12" s="10" t="str">
         <x:f>IF(M12="","",LOWER(M12))</x:f>
       </x:c>
+      <x:c r="O12" s="4"/>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="11"/>
@@ -616,11 +631,12 @@
       <x:c r="K13" s="9"/>
       <x:c r="L13" s="9"/>
       <x:c r="M13" s="10" t="str">
-        <x:f>IF(A13="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O13&lt;&gt;"",O13,IF(A13="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N13" s="10" t="str">
         <x:f>IF(M13="","",LOWER(M13))</x:f>
       </x:c>
+      <x:c r="O13" s="4"/>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="11"/>
@@ -636,11 +652,12 @@
       <x:c r="K14" s="9"/>
       <x:c r="L14" s="9"/>
       <x:c r="M14" s="10" t="str">
-        <x:f>IF(A14="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O14&lt;&gt;"",O14,IF(A14="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N14" s="10" t="str">
         <x:f>IF(M14="","",LOWER(M14))</x:f>
       </x:c>
+      <x:c r="O14" s="4"/>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="11"/>
@@ -656,11 +673,12 @@
       <x:c r="K15" s="9"/>
       <x:c r="L15" s="9"/>
       <x:c r="M15" s="10" t="str">
-        <x:f>IF(A15="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O15&lt;&gt;"",O15,IF(A15="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N15" s="10" t="str">
         <x:f>IF(M15="","",LOWER(M15))</x:f>
       </x:c>
+      <x:c r="O15" s="4"/>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="11"/>
@@ -676,11 +694,12 @@
       <x:c r="K16" s="9"/>
       <x:c r="L16" s="9"/>
       <x:c r="M16" s="10" t="str">
-        <x:f>IF(A16="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O16&lt;&gt;"",O16,IF(A16="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N16" s="10" t="str">
         <x:f>IF(M16="","",LOWER(M16))</x:f>
       </x:c>
+      <x:c r="O16" s="4"/>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="11"/>
@@ -696,11 +715,12 @@
       <x:c r="K17" s="9"/>
       <x:c r="L17" s="9"/>
       <x:c r="M17" s="10" t="str">
-        <x:f>IF(A17="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O17&lt;&gt;"",O17,IF(A17="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N17" s="10" t="str">
         <x:f>IF(M17="","",LOWER(M17))</x:f>
       </x:c>
+      <x:c r="O17" s="4"/>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="11"/>
@@ -716,11 +736,12 @@
       <x:c r="K18" s="9"/>
       <x:c r="L18" s="9"/>
       <x:c r="M18" s="10" t="str">
-        <x:f>IF(A18="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O18&lt;&gt;"",O18,IF(A18="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N18" s="10" t="str">
         <x:f>IF(M18="","",LOWER(M18))</x:f>
       </x:c>
+      <x:c r="O18" s="4"/>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="11"/>
@@ -736,11 +757,12 @@
       <x:c r="K19" s="9"/>
       <x:c r="L19" s="9"/>
       <x:c r="M19" s="10" t="str">
-        <x:f>IF(A19="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O19&lt;&gt;"",O19,IF(A19="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N19" s="10" t="str">
         <x:f>IF(M19="","",LOWER(M19))</x:f>
       </x:c>
+      <x:c r="O19" s="4"/>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="11"/>
@@ -756,11 +778,12 @@
       <x:c r="K20" s="9"/>
       <x:c r="L20" s="9"/>
       <x:c r="M20" s="10" t="str">
-        <x:f>IF(A20="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O20&lt;&gt;"",O20,IF(A20="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N20" s="10" t="str">
         <x:f>IF(M20="","",LOWER(M20))</x:f>
       </x:c>
+      <x:c r="O20" s="4"/>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="11"/>
@@ -776,11 +799,12 @@
       <x:c r="K21" s="9"/>
       <x:c r="L21" s="9"/>
       <x:c r="M21" s="10" t="str">
-        <x:f>IF(A21="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O21&lt;&gt;"",O21,IF(A21="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N21" s="10" t="str">
         <x:f>IF(M21="","",LOWER(M21))</x:f>
       </x:c>
+      <x:c r="O21" s="4"/>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="11"/>
@@ -796,11 +820,12 @@
       <x:c r="K22" s="9"/>
       <x:c r="L22" s="9"/>
       <x:c r="M22" s="10" t="str">
-        <x:f>IF(A22="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O22&lt;&gt;"",O22,IF(A22="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N22" s="10" t="str">
         <x:f>IF(M22="","",LOWER(M22))</x:f>
       </x:c>
+      <x:c r="O22" s="4"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="11"/>
@@ -816,11 +841,12 @@
       <x:c r="K23" s="9"/>
       <x:c r="L23" s="9"/>
       <x:c r="M23" s="10" t="str">
-        <x:f>IF(A23="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O23&lt;&gt;"",O23,IF(A23="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N23" s="10" t="str">
         <x:f>IF(M23="","",LOWER(M23))</x:f>
       </x:c>
+      <x:c r="O23" s="4"/>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="11"/>
@@ -836,11 +862,12 @@
       <x:c r="K24" s="9"/>
       <x:c r="L24" s="9"/>
       <x:c r="M24" s="10" t="str">
-        <x:f>IF(A24="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O24&lt;&gt;"",O24,IF(A24="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N24" s="10" t="str">
         <x:f>IF(M24="","",LOWER(M24))</x:f>
       </x:c>
+      <x:c r="O24" s="4"/>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="11"/>
@@ -856,11 +883,12 @@
       <x:c r="K25" s="9"/>
       <x:c r="L25" s="9"/>
       <x:c r="M25" s="10" t="str">
-        <x:f>IF(A25="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O25&lt;&gt;"",O25,IF(A25="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N25" s="10" t="str">
         <x:f>IF(M25="","",LOWER(M25))</x:f>
       </x:c>
+      <x:c r="O25" s="4"/>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="11"/>
@@ -876,11 +904,12 @@
       <x:c r="K26" s="9"/>
       <x:c r="L26" s="9"/>
       <x:c r="M26" s="10" t="str">
-        <x:f>IF(A26="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O26&lt;&gt;"",O26,IF(A26="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N26" s="10" t="str">
         <x:f>IF(M26="","",LOWER(M26))</x:f>
       </x:c>
+      <x:c r="O26" s="4"/>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="11"/>
@@ -896,11 +925,12 @@
       <x:c r="K27" s="9"/>
       <x:c r="L27" s="9"/>
       <x:c r="M27" s="10" t="str">
-        <x:f>IF(A27="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O27&lt;&gt;"",O27,IF(A27="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N27" s="10" t="str">
         <x:f>IF(M27="","",LOWER(M27))</x:f>
       </x:c>
+      <x:c r="O27" s="4"/>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="11"/>
@@ -916,11 +946,12 @@
       <x:c r="K28" s="9"/>
       <x:c r="L28" s="9"/>
       <x:c r="M28" s="10" t="str">
-        <x:f>IF(A28="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O28&lt;&gt;"",O28,IF(A28="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N28" s="10" t="str">
         <x:f>IF(M28="","",LOWER(M28))</x:f>
       </x:c>
+      <x:c r="O28" s="4"/>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="11"/>
@@ -936,11 +967,12 @@
       <x:c r="K29" s="9"/>
       <x:c r="L29" s="9"/>
       <x:c r="M29" s="10" t="str">
-        <x:f>IF(A29="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O29&lt;&gt;"",O29,IF(A29="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N29" s="10" t="str">
         <x:f>IF(M29="","",LOWER(M29))</x:f>
       </x:c>
+      <x:c r="O29" s="4"/>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="11"/>
@@ -956,11 +988,12 @@
       <x:c r="K30" s="9"/>
       <x:c r="L30" s="9"/>
       <x:c r="M30" s="10" t="str">
-        <x:f>IF(A30="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O30&lt;&gt;"",O30,IF(A30="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N30" s="10" t="str">
         <x:f>IF(M30="","",LOWER(M30))</x:f>
       </x:c>
+      <x:c r="O30" s="4"/>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="11"/>
@@ -976,11 +1009,12 @@
       <x:c r="K31" s="9"/>
       <x:c r="L31" s="9"/>
       <x:c r="M31" s="10" t="str">
-        <x:f>IF(A31="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O31&lt;&gt;"",O31,IF(A31="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N31" s="10" t="str">
         <x:f>IF(M31="","",LOWER(M31))</x:f>
       </x:c>
+      <x:c r="O31" s="4"/>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="11"/>
@@ -996,11 +1030,12 @@
       <x:c r="K32" s="9"/>
       <x:c r="L32" s="9"/>
       <x:c r="M32" s="10" t="str">
-        <x:f>IF(A32="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O32&lt;&gt;"",O32,IF(A32="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N32" s="10" t="str">
         <x:f>IF(M32="","",LOWER(M32))</x:f>
       </x:c>
+      <x:c r="O32" s="4"/>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="11"/>
@@ -1016,11 +1051,12 @@
       <x:c r="K33" s="9"/>
       <x:c r="L33" s="9"/>
       <x:c r="M33" s="10" t="str">
-        <x:f>IF(A33="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O33&lt;&gt;"",O33,IF(A33="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N33" s="10" t="str">
         <x:f>IF(M33="","",LOWER(M33))</x:f>
       </x:c>
+      <x:c r="O33" s="4"/>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="11"/>
@@ -1036,11 +1072,12 @@
       <x:c r="K34" s="9"/>
       <x:c r="L34" s="9"/>
       <x:c r="M34" s="10" t="str">
-        <x:f>IF(A34="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O34&lt;&gt;"",O34,IF(A34="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N34" s="10" t="str">
         <x:f>IF(M34="","",LOWER(M34))</x:f>
       </x:c>
+      <x:c r="O34" s="4"/>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="11"/>
@@ -1056,11 +1093,12 @@
       <x:c r="K35" s="9"/>
       <x:c r="L35" s="9"/>
       <x:c r="M35" s="10" t="str">
-        <x:f>IF(A35="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O35&lt;&gt;"",O35,IF(A35="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N35" s="10" t="str">
         <x:f>IF(M35="","",LOWER(M35))</x:f>
       </x:c>
+      <x:c r="O35" s="4"/>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="11"/>
@@ -1076,11 +1114,12 @@
       <x:c r="K36" s="9"/>
       <x:c r="L36" s="9"/>
       <x:c r="M36" s="10" t="str">
-        <x:f>IF(A36="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O36&lt;&gt;"",O36,IF(A36="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N36" s="10" t="str">
         <x:f>IF(M36="","",LOWER(M36))</x:f>
       </x:c>
+      <x:c r="O36" s="4"/>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="11"/>
@@ -1096,11 +1135,12 @@
       <x:c r="K37" s="9"/>
       <x:c r="L37" s="9"/>
       <x:c r="M37" s="10" t="str">
-        <x:f>IF(A37="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O37&lt;&gt;"",O37,IF(A37="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N37" s="10" t="str">
         <x:f>IF(M37="","",LOWER(M37))</x:f>
       </x:c>
+      <x:c r="O37" s="4"/>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="11"/>
@@ -1116,11 +1156,12 @@
       <x:c r="K38" s="9"/>
       <x:c r="L38" s="9"/>
       <x:c r="M38" s="10" t="str">
-        <x:f>IF(A38="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O38&lt;&gt;"",O38,IF(A38="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N38" s="10" t="str">
         <x:f>IF(M38="","",LOWER(M38))</x:f>
       </x:c>
+      <x:c r="O38" s="4"/>
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="11"/>
@@ -1136,11 +1177,12 @@
       <x:c r="K39" s="9"/>
       <x:c r="L39" s="9"/>
       <x:c r="M39" s="10" t="str">
-        <x:f>IF(A39="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O39&lt;&gt;"",O39,IF(A39="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N39" s="10" t="str">
         <x:f>IF(M39="","",LOWER(M39))</x:f>
       </x:c>
+      <x:c r="O39" s="4"/>
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="11"/>
@@ -1156,11 +1198,12 @@
       <x:c r="K40" s="9"/>
       <x:c r="L40" s="9"/>
       <x:c r="M40" s="10" t="str">
-        <x:f>IF(A40="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O40&lt;&gt;"",O40,IF(A40="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N40" s="10" t="str">
         <x:f>IF(M40="","",LOWER(M40))</x:f>
       </x:c>
+      <x:c r="O40" s="4"/>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="11"/>
@@ -1176,11 +1219,12 @@
       <x:c r="K41" s="9"/>
       <x:c r="L41" s="9"/>
       <x:c r="M41" s="10" t="str">
-        <x:f>IF(A41="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O41&lt;&gt;"",O41,IF(A41="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N41" s="10" t="str">
         <x:f>IF(M41="","",LOWER(M41))</x:f>
       </x:c>
+      <x:c r="O41" s="4"/>
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" s="11"/>
@@ -1196,11 +1240,12 @@
       <x:c r="K42" s="9"/>
       <x:c r="L42" s="9"/>
       <x:c r="M42" s="10" t="str">
-        <x:f>IF(A42="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O42&lt;&gt;"",O42,IF(A42="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N42" s="10" t="str">
         <x:f>IF(M42="","",LOWER(M42))</x:f>
       </x:c>
+      <x:c r="O42" s="4"/>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="11"/>
@@ -1216,11 +1261,12 @@
       <x:c r="K43" s="9"/>
       <x:c r="L43" s="9"/>
       <x:c r="M43" s="10" t="str">
-        <x:f>IF(A43="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O43&lt;&gt;"",O43,IF(A43="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N43" s="10" t="str">
         <x:f>IF(M43="","",LOWER(M43))</x:f>
       </x:c>
+      <x:c r="O43" s="4"/>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="11"/>
@@ -1236,11 +1282,12 @@
       <x:c r="K44" s="9"/>
       <x:c r="L44" s="9"/>
       <x:c r="M44" s="10" t="str">
-        <x:f>IF(A44="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O44&lt;&gt;"",O44,IF(A44="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N44" s="10" t="str">
         <x:f>IF(M44="","",LOWER(M44))</x:f>
       </x:c>
+      <x:c r="O44" s="4"/>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" s="11"/>
@@ -1256,11 +1303,12 @@
       <x:c r="K45" s="9"/>
       <x:c r="L45" s="9"/>
       <x:c r="M45" s="10" t="str">
-        <x:f>IF(A45="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O45&lt;&gt;"",O45,IF(A45="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N45" s="10" t="str">
         <x:f>IF(M45="","",LOWER(M45))</x:f>
       </x:c>
+      <x:c r="O45" s="4"/>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" s="11"/>
@@ -1276,11 +1324,12 @@
       <x:c r="K46" s="9"/>
       <x:c r="L46" s="9"/>
       <x:c r="M46" s="10" t="str">
-        <x:f>IF(A46="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O46&lt;&gt;"",O46,IF(A46="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N46" s="10" t="str">
         <x:f>IF(M46="","",LOWER(M46))</x:f>
       </x:c>
+      <x:c r="O46" s="4"/>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" s="11"/>
@@ -1296,11 +1345,12 @@
       <x:c r="K47" s="9"/>
       <x:c r="L47" s="9"/>
       <x:c r="M47" s="10" t="str">
-        <x:f>IF(A47="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O47&lt;&gt;"",O47,IF(A47="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N47" s="10" t="str">
         <x:f>IF(M47="","",LOWER(M47))</x:f>
       </x:c>
+      <x:c r="O47" s="4"/>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" s="11"/>
@@ -1316,11 +1366,12 @@
       <x:c r="K48" s="9"/>
       <x:c r="L48" s="9"/>
       <x:c r="M48" s="10" t="str">
-        <x:f>IF(A48="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O48&lt;&gt;"",O48,IF(A48="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N48" s="10" t="str">
         <x:f>IF(M48="","",LOWER(M48))</x:f>
       </x:c>
+      <x:c r="O48" s="4"/>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" s="11"/>
@@ -1336,11 +1387,12 @@
       <x:c r="K49" s="9"/>
       <x:c r="L49" s="9"/>
       <x:c r="M49" s="10" t="str">
-        <x:f>IF(A49="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O49&lt;&gt;"",O49,IF(A49="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N49" s="10" t="str">
         <x:f>IF(M49="","",LOWER(M49))</x:f>
       </x:c>
+      <x:c r="O49" s="4"/>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" s="11"/>
@@ -1356,11 +1408,12 @@
       <x:c r="K50" s="9"/>
       <x:c r="L50" s="9"/>
       <x:c r="M50" s="10" t="str">
-        <x:f>IF(A50="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O50&lt;&gt;"",O50,IF(A50="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N50" s="10" t="str">
         <x:f>IF(M50="","",LOWER(M50))</x:f>
       </x:c>
+      <x:c r="O50" s="4"/>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" s="11"/>
@@ -1376,11 +1429,12 @@
       <x:c r="K51" s="9"/>
       <x:c r="L51" s="9"/>
       <x:c r="M51" s="10" t="str">
-        <x:f>IF(A51="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O51&lt;&gt;"",O51,IF(A51="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N51" s="10" t="str">
         <x:f>IF(M51="","",LOWER(M51))</x:f>
       </x:c>
+      <x:c r="O51" s="4"/>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" s="11"/>
@@ -1396,11 +1450,12 @@
       <x:c r="K52" s="9"/>
       <x:c r="L52" s="9"/>
       <x:c r="M52" s="10" t="str">
-        <x:f>IF(A52="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O52&lt;&gt;"",O52,IF(A52="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N52" s="10" t="str">
         <x:f>IF(M52="","",LOWER(M52))</x:f>
       </x:c>
+      <x:c r="O52" s="4"/>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" s="11"/>
@@ -1416,11 +1471,12 @@
       <x:c r="K53" s="9"/>
       <x:c r="L53" s="9"/>
       <x:c r="M53" s="10" t="str">
-        <x:f>IF(A53="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O53&lt;&gt;"",O53,IF(A53="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N53" s="10" t="str">
         <x:f>IF(M53="","",LOWER(M53))</x:f>
       </x:c>
+      <x:c r="O53" s="4"/>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" s="11"/>
@@ -1436,11 +1492,12 @@
       <x:c r="K54" s="9"/>
       <x:c r="L54" s="9"/>
       <x:c r="M54" s="10" t="str">
-        <x:f>IF(A54="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O54&lt;&gt;"",O54,IF(A54="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N54" s="10" t="str">
         <x:f>IF(M54="","",LOWER(M54))</x:f>
       </x:c>
+      <x:c r="O54" s="4"/>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" s="11"/>
@@ -1456,11 +1513,12 @@
       <x:c r="K55" s="9"/>
       <x:c r="L55" s="9"/>
       <x:c r="M55" s="10" t="str">
-        <x:f>IF(A55="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O55&lt;&gt;"",O55,IF(A55="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N55" s="10" t="str">
         <x:f>IF(M55="","",LOWER(M55))</x:f>
       </x:c>
+      <x:c r="O55" s="4"/>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" s="11"/>
@@ -1476,11 +1534,12 @@
       <x:c r="K56" s="9"/>
       <x:c r="L56" s="9"/>
       <x:c r="M56" s="10" t="str">
-        <x:f>IF(A56="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O56&lt;&gt;"",O56,IF(A56="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N56" s="10" t="str">
         <x:f>IF(M56="","",LOWER(M56))</x:f>
       </x:c>
+      <x:c r="O56" s="4"/>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" s="11"/>
@@ -1496,11 +1555,12 @@
       <x:c r="K57" s="9"/>
       <x:c r="L57" s="9"/>
       <x:c r="M57" s="10" t="str">
-        <x:f>IF(A57="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O57&lt;&gt;"",O57,IF(A57="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N57" s="10" t="str">
         <x:f>IF(M57="","",LOWER(M57))</x:f>
       </x:c>
+      <x:c r="O57" s="4"/>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" s="11"/>
@@ -1516,11 +1576,12 @@
       <x:c r="K58" s="9"/>
       <x:c r="L58" s="9"/>
       <x:c r="M58" s="10" t="str">
-        <x:f>IF(A58="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O58&lt;&gt;"",O58,IF(A58="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N58" s="10" t="str">
         <x:f>IF(M58="","",LOWER(M58))</x:f>
       </x:c>
+      <x:c r="O58" s="4"/>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" s="11"/>
@@ -1536,11 +1597,12 @@
       <x:c r="K59" s="9"/>
       <x:c r="L59" s="9"/>
       <x:c r="M59" s="10" t="str">
-        <x:f>IF(A59="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O59&lt;&gt;"",O59,IF(A59="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N59" s="10" t="str">
         <x:f>IF(M59="","",LOWER(M59))</x:f>
       </x:c>
+      <x:c r="O59" s="4"/>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" s="11"/>
@@ -1556,11 +1618,12 @@
       <x:c r="K60" s="9"/>
       <x:c r="L60" s="9"/>
       <x:c r="M60" s="10" t="str">
-        <x:f>IF(A60="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O60&lt;&gt;"",O60,IF(A60="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N60" s="10" t="str">
         <x:f>IF(M60="","",LOWER(M60))</x:f>
       </x:c>
+      <x:c r="O60" s="4"/>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" s="11"/>
@@ -1576,11 +1639,12 @@
       <x:c r="K61" s="9"/>
       <x:c r="L61" s="9"/>
       <x:c r="M61" s="10" t="str">
-        <x:f>IF(A61="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O61&lt;&gt;"",O61,IF(A61="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N61" s="10" t="str">
         <x:f>IF(M61="","",LOWER(M61))</x:f>
       </x:c>
+      <x:c r="O61" s="4"/>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" s="11"/>
@@ -1596,11 +1660,12 @@
       <x:c r="K62" s="9"/>
       <x:c r="L62" s="9"/>
       <x:c r="M62" s="10" t="str">
-        <x:f>IF(A62="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O62&lt;&gt;"",O62,IF(A62="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N62" s="10" t="str">
         <x:f>IF(M62="","",LOWER(M62))</x:f>
       </x:c>
+      <x:c r="O62" s="4"/>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" s="11"/>
@@ -1616,11 +1681,12 @@
       <x:c r="K63" s="9"/>
       <x:c r="L63" s="9"/>
       <x:c r="M63" s="10" t="str">
-        <x:f>IF(A63="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O63&lt;&gt;"",O63,IF(A63="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N63" s="10" t="str">
         <x:f>IF(M63="","",LOWER(M63))</x:f>
       </x:c>
+      <x:c r="O63" s="4"/>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" s="11"/>
@@ -1636,11 +1702,12 @@
       <x:c r="K64" s="9"/>
       <x:c r="L64" s="9"/>
       <x:c r="M64" s="10" t="str">
-        <x:f>IF(A64="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O64&lt;&gt;"",O64,IF(A64="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N64" s="10" t="str">
         <x:f>IF(M64="","",LOWER(M64))</x:f>
       </x:c>
+      <x:c r="O64" s="4"/>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" s="11"/>
@@ -1656,11 +1723,12 @@
       <x:c r="K65" s="9"/>
       <x:c r="L65" s="9"/>
       <x:c r="M65" s="10" t="str">
-        <x:f>IF(A65="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O65&lt;&gt;"",O65,IF(A65="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N65" s="10" t="str">
         <x:f>IF(M65="","",LOWER(M65))</x:f>
       </x:c>
+      <x:c r="O65" s="4"/>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" s="11"/>
@@ -1676,11 +1744,12 @@
       <x:c r="K66" s="9"/>
       <x:c r="L66" s="9"/>
       <x:c r="M66" s="10" t="str">
-        <x:f>IF(A66="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O66&lt;&gt;"",O66,IF(A66="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N66" s="10" t="str">
         <x:f>IF(M66="","",LOWER(M66))</x:f>
       </x:c>
+      <x:c r="O66" s="4"/>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" s="11"/>
@@ -1696,11 +1765,12 @@
       <x:c r="K67" s="9"/>
       <x:c r="L67" s="9"/>
       <x:c r="M67" s="10" t="str">
-        <x:f>IF(A67="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O67&lt;&gt;"",O67,IF(A67="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N67" s="10" t="str">
         <x:f>IF(M67="","",LOWER(M67))</x:f>
       </x:c>
+      <x:c r="O67" s="4"/>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" s="11"/>
@@ -1716,11 +1786,12 @@
       <x:c r="K68" s="9"/>
       <x:c r="L68" s="9"/>
       <x:c r="M68" s="10" t="str">
-        <x:f>IF(A68="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O68&lt;&gt;"",O68,IF(A68="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N68" s="10" t="str">
         <x:f>IF(M68="","",LOWER(M68))</x:f>
       </x:c>
+      <x:c r="O68" s="4"/>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" s="11"/>
@@ -1736,11 +1807,12 @@
       <x:c r="K69" s="9"/>
       <x:c r="L69" s="9"/>
       <x:c r="M69" s="10" t="str">
-        <x:f>IF(A69="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O69&lt;&gt;"",O69,IF(A69="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N69" s="10" t="str">
         <x:f>IF(M69="","",LOWER(M69))</x:f>
       </x:c>
+      <x:c r="O69" s="4"/>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" s="11"/>
@@ -1756,11 +1828,12 @@
       <x:c r="K70" s="9"/>
       <x:c r="L70" s="9"/>
       <x:c r="M70" s="10" t="str">
-        <x:f>IF(A70="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O70&lt;&gt;"",O70,IF(A70="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N70" s="10" t="str">
         <x:f>IF(M70="","",LOWER(M70))</x:f>
       </x:c>
+      <x:c r="O70" s="4"/>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" s="11"/>
@@ -1776,11 +1849,12 @@
       <x:c r="K71" s="9"/>
       <x:c r="L71" s="9"/>
       <x:c r="M71" s="10" t="str">
-        <x:f>IF(A71="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O71&lt;&gt;"",O71,IF(A71="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N71" s="10" t="str">
         <x:f>IF(M71="","",LOWER(M71))</x:f>
       </x:c>
+      <x:c r="O71" s="4"/>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" s="11"/>
@@ -1796,11 +1870,12 @@
       <x:c r="K72" s="9"/>
       <x:c r="L72" s="9"/>
       <x:c r="M72" s="10" t="str">
-        <x:f>IF(A72="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O72&lt;&gt;"",O72,IF(A72="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N72" s="10" t="str">
         <x:f>IF(M72="","",LOWER(M72))</x:f>
       </x:c>
+      <x:c r="O72" s="4"/>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" s="11"/>
@@ -1816,11 +1891,12 @@
       <x:c r="K73" s="9"/>
       <x:c r="L73" s="9"/>
       <x:c r="M73" s="10" t="str">
-        <x:f>IF(A73="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O73&lt;&gt;"",O73,IF(A73="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N73" s="10" t="str">
         <x:f>IF(M73="","",LOWER(M73))</x:f>
       </x:c>
+      <x:c r="O73" s="4"/>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" s="11"/>
@@ -1836,11 +1912,12 @@
       <x:c r="K74" s="9"/>
       <x:c r="L74" s="9"/>
       <x:c r="M74" s="10" t="str">
-        <x:f>IF(A74="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O74&lt;&gt;"",O74,IF(A74="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N74" s="10" t="str">
         <x:f>IF(M74="","",LOWER(M74))</x:f>
       </x:c>
+      <x:c r="O74" s="4"/>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" s="11"/>
@@ -1856,11 +1933,12 @@
       <x:c r="K75" s="9"/>
       <x:c r="L75" s="9"/>
       <x:c r="M75" s="10" t="str">
-        <x:f>IF(A75="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O75&lt;&gt;"",O75,IF(A75="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N75" s="10" t="str">
         <x:f>IF(M75="","",LOWER(M75))</x:f>
       </x:c>
+      <x:c r="O75" s="4"/>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" s="11"/>
@@ -1876,11 +1954,12 @@
       <x:c r="K76" s="9"/>
       <x:c r="L76" s="9"/>
       <x:c r="M76" s="10" t="str">
-        <x:f>IF(A76="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O76&lt;&gt;"",O76,IF(A76="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N76" s="10" t="str">
         <x:f>IF(M76="","",LOWER(M76))</x:f>
       </x:c>
+      <x:c r="O76" s="4"/>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" s="11"/>
@@ -1896,11 +1975,12 @@
       <x:c r="K77" s="9"/>
       <x:c r="L77" s="9"/>
       <x:c r="M77" s="10" t="str">
-        <x:f>IF(A77="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O77&lt;&gt;"",O77,IF(A77="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N77" s="10" t="str">
         <x:f>IF(M77="","",LOWER(M77))</x:f>
       </x:c>
+      <x:c r="O77" s="4"/>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" s="11"/>
@@ -1916,11 +1996,12 @@
       <x:c r="K78" s="9"/>
       <x:c r="L78" s="9"/>
       <x:c r="M78" s="10" t="str">
-        <x:f>IF(A78="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O78&lt;&gt;"",O78,IF(A78="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N78" s="10" t="str">
         <x:f>IF(M78="","",LOWER(M78))</x:f>
       </x:c>
+      <x:c r="O78" s="4"/>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" s="11"/>
@@ -1936,11 +2017,12 @@
       <x:c r="K79" s="9"/>
       <x:c r="L79" s="9"/>
       <x:c r="M79" s="10" t="str">
-        <x:f>IF(A79="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O79&lt;&gt;"",O79,IF(A79="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N79" s="10" t="str">
         <x:f>IF(M79="","",LOWER(M79))</x:f>
       </x:c>
+      <x:c r="O79" s="4"/>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" s="11"/>
@@ -1956,11 +2038,12 @@
       <x:c r="K80" s="9"/>
       <x:c r="L80" s="9"/>
       <x:c r="M80" s="10" t="str">
-        <x:f>IF(A80="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O80&lt;&gt;"",O80,IF(A80="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N80" s="10" t="str">
         <x:f>IF(M80="","",LOWER(M80))</x:f>
       </x:c>
+      <x:c r="O80" s="4"/>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" s="11"/>
@@ -1976,11 +2059,12 @@
       <x:c r="K81" s="9"/>
       <x:c r="L81" s="9"/>
       <x:c r="M81" s="10" t="str">
-        <x:f>IF(A81="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O81&lt;&gt;"",O81,IF(A81="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N81" s="10" t="str">
         <x:f>IF(M81="","",LOWER(M81))</x:f>
       </x:c>
+      <x:c r="O81" s="4"/>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" s="11"/>
@@ -1996,11 +2080,12 @@
       <x:c r="K82" s="9"/>
       <x:c r="L82" s="9"/>
       <x:c r="M82" s="10" t="str">
-        <x:f>IF(A82="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O82&lt;&gt;"",O82,IF(A82="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N82" s="10" t="str">
         <x:f>IF(M82="","",LOWER(M82))</x:f>
       </x:c>
+      <x:c r="O82" s="4"/>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" s="11"/>
@@ -2016,11 +2101,12 @@
       <x:c r="K83" s="9"/>
       <x:c r="L83" s="9"/>
       <x:c r="M83" s="10" t="str">
-        <x:f>IF(A83="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O83&lt;&gt;"",O83,IF(A83="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N83" s="10" t="str">
         <x:f>IF(M83="","",LOWER(M83))</x:f>
       </x:c>
+      <x:c r="O83" s="4"/>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" s="11"/>
@@ -2036,11 +2122,12 @@
       <x:c r="K84" s="9"/>
       <x:c r="L84" s="9"/>
       <x:c r="M84" s="10" t="str">
-        <x:f>IF(A84="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O84&lt;&gt;"",O84,IF(A84="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N84" s="10" t="str">
         <x:f>IF(M84="","",LOWER(M84))</x:f>
       </x:c>
+      <x:c r="O84" s="4"/>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" s="11"/>
@@ -2056,11 +2143,12 @@
       <x:c r="K85" s="9"/>
       <x:c r="L85" s="9"/>
       <x:c r="M85" s="10" t="str">
-        <x:f>IF(A85="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O85&lt;&gt;"",O85,IF(A85="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N85" s="10" t="str">
         <x:f>IF(M85="","",LOWER(M85))</x:f>
       </x:c>
+      <x:c r="O85" s="4"/>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" s="11"/>
@@ -2076,11 +2164,12 @@
       <x:c r="K86" s="9"/>
       <x:c r="L86" s="9"/>
       <x:c r="M86" s="10" t="str">
-        <x:f>IF(A86="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O86&lt;&gt;"",O86,IF(A86="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N86" s="10" t="str">
         <x:f>IF(M86="","",LOWER(M86))</x:f>
       </x:c>
+      <x:c r="O86" s="4"/>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" s="11"/>
@@ -2096,11 +2185,12 @@
       <x:c r="K87" s="9"/>
       <x:c r="L87" s="9"/>
       <x:c r="M87" s="10" t="str">
-        <x:f>IF(A87="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O87&lt;&gt;"",O87,IF(A87="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N87" s="10" t="str">
         <x:f>IF(M87="","",LOWER(M87))</x:f>
       </x:c>
+      <x:c r="O87" s="4"/>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" s="11"/>
@@ -2116,11 +2206,12 @@
       <x:c r="K88" s="9"/>
       <x:c r="L88" s="9"/>
       <x:c r="M88" s="10" t="str">
-        <x:f>IF(A88="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O88&lt;&gt;"",O88,IF(A88="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N88" s="10" t="str">
         <x:f>IF(M88="","",LOWER(M88))</x:f>
       </x:c>
+      <x:c r="O88" s="4"/>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" s="11"/>
@@ -2136,11 +2227,12 @@
       <x:c r="K89" s="9"/>
       <x:c r="L89" s="9"/>
       <x:c r="M89" s="10" t="str">
-        <x:f>IF(A89="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O89&lt;&gt;"",O89,IF(A89="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N89" s="10" t="str">
         <x:f>IF(M89="","",LOWER(M89))</x:f>
       </x:c>
+      <x:c r="O89" s="4"/>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" s="11"/>
@@ -2156,11 +2248,12 @@
       <x:c r="K90" s="9"/>
       <x:c r="L90" s="9"/>
       <x:c r="M90" s="10" t="str">
-        <x:f>IF(A90="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O90&lt;&gt;"",O90,IF(A90="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N90" s="10" t="str">
         <x:f>IF(M90="","",LOWER(M90))</x:f>
       </x:c>
+      <x:c r="O90" s="4"/>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" s="11"/>
@@ -2176,11 +2269,12 @@
       <x:c r="K91" s="9"/>
       <x:c r="L91" s="9"/>
       <x:c r="M91" s="10" t="str">
-        <x:f>IF(A91="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O91&lt;&gt;"",O91,IF(A91="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N91" s="10" t="str">
         <x:f>IF(M91="","",LOWER(M91))</x:f>
       </x:c>
+      <x:c r="O91" s="4"/>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" s="11"/>
@@ -2196,11 +2290,12 @@
       <x:c r="K92" s="9"/>
       <x:c r="L92" s="9"/>
       <x:c r="M92" s="10" t="str">
-        <x:f>IF(A92="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O92&lt;&gt;"",O92,IF(A92="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N92" s="10" t="str">
         <x:f>IF(M92="","",LOWER(M92))</x:f>
       </x:c>
+      <x:c r="O92" s="4"/>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" s="11"/>
@@ -2216,11 +2311,12 @@
       <x:c r="K93" s="9"/>
       <x:c r="L93" s="9"/>
       <x:c r="M93" s="10" t="str">
-        <x:f>IF(A93="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O93&lt;&gt;"",O93,IF(A93="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N93" s="10" t="str">
         <x:f>IF(M93="","",LOWER(M93))</x:f>
       </x:c>
+      <x:c r="O93" s="4"/>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" s="11"/>
@@ -2236,11 +2332,12 @@
       <x:c r="K94" s="9"/>
       <x:c r="L94" s="9"/>
       <x:c r="M94" s="10" t="str">
-        <x:f>IF(A94="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O94&lt;&gt;"",O94,IF(A94="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N94" s="10" t="str">
         <x:f>IF(M94="","",LOWER(M94))</x:f>
       </x:c>
+      <x:c r="O94" s="4"/>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" s="11"/>
@@ -2256,11 +2353,12 @@
       <x:c r="K95" s="9"/>
       <x:c r="L95" s="9"/>
       <x:c r="M95" s="10" t="str">
-        <x:f>IF(A95="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O95&lt;&gt;"",O95,IF(A95="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N95" s="10" t="str">
         <x:f>IF(M95="","",LOWER(M95))</x:f>
       </x:c>
+      <x:c r="O95" s="4"/>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" s="11"/>
@@ -2276,11 +2374,12 @@
       <x:c r="K96" s="9"/>
       <x:c r="L96" s="9"/>
       <x:c r="M96" s="10" t="str">
-        <x:f>IF(A96="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O96&lt;&gt;"",O96,IF(A96="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N96" s="10" t="str">
         <x:f>IF(M96="","",LOWER(M96))</x:f>
       </x:c>
+      <x:c r="O96" s="4"/>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" s="11"/>
@@ -2296,11 +2395,12 @@
       <x:c r="K97" s="9"/>
       <x:c r="L97" s="9"/>
       <x:c r="M97" s="10" t="str">
-        <x:f>IF(A97="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O97&lt;&gt;"",O97,IF(A97="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N97" s="10" t="str">
         <x:f>IF(M97="","",LOWER(M97))</x:f>
       </x:c>
+      <x:c r="O97" s="4"/>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" s="11"/>
@@ -2316,11 +2416,12 @@
       <x:c r="K98" s="9"/>
       <x:c r="L98" s="9"/>
       <x:c r="M98" s="10" t="str">
-        <x:f>IF(A98="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O98&lt;&gt;"",O98,IF(A98="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N98" s="10" t="str">
         <x:f>IF(M98="","",LOWER(M98))</x:f>
       </x:c>
+      <x:c r="O98" s="4"/>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" s="11"/>
@@ -2336,11 +2437,12 @@
       <x:c r="K99" s="9"/>
       <x:c r="L99" s="9"/>
       <x:c r="M99" s="10" t="str">
-        <x:f>IF(A99="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O99&lt;&gt;"",O99,IF(A99="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N99" s="10" t="str">
         <x:f>IF(M99="","",LOWER(M99))</x:f>
       </x:c>
+      <x:c r="O99" s="4"/>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" s="11"/>
@@ -2356,11 +2458,12 @@
       <x:c r="K100" s="9"/>
       <x:c r="L100" s="9"/>
       <x:c r="M100" s="10" t="str">
-        <x:f>IF(A100="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O100&lt;&gt;"",O100,IF(A100="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N100" s="10" t="str">
         <x:f>IF(M100="","",LOWER(M100))</x:f>
       </x:c>
+      <x:c r="O100" s="4"/>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" s="11"/>
@@ -2376,11 +2479,12 @@
       <x:c r="K101" s="9"/>
       <x:c r="L101" s="9"/>
       <x:c r="M101" s="10" t="str">
-        <x:f>IF(A101="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O101&lt;&gt;"",O101,IF(A101="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N101" s="10" t="str">
         <x:f>IF(M101="","",LOWER(M101))</x:f>
       </x:c>
+      <x:c r="O101" s="4"/>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" s="11"/>
@@ -2396,11 +2500,12 @@
       <x:c r="K102" s="9"/>
       <x:c r="L102" s="9"/>
       <x:c r="M102" s="10" t="str">
-        <x:f>IF(A102="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O102&lt;&gt;"",O102,IF(A102="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N102" s="10" t="str">
         <x:f>IF(M102="","",LOWER(M102))</x:f>
       </x:c>
+      <x:c r="O102" s="4"/>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" s="11"/>
@@ -2416,11 +2521,12 @@
       <x:c r="K103" s="9"/>
       <x:c r="L103" s="9"/>
       <x:c r="M103" s="10" t="str">
-        <x:f>IF(A103="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O103&lt;&gt;"",O103,IF(A103="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N103" s="10" t="str">
         <x:f>IF(M103="","",LOWER(M103))</x:f>
       </x:c>
+      <x:c r="O103" s="4"/>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" s="11"/>
@@ -2436,11 +2542,12 @@
       <x:c r="K104" s="9"/>
       <x:c r="L104" s="9"/>
       <x:c r="M104" s="10" t="str">
-        <x:f>IF(A104="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O104&lt;&gt;"",O104,IF(A104="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N104" s="10" t="str">
         <x:f>IF(M104="","",LOWER(M104))</x:f>
       </x:c>
+      <x:c r="O104" s="4"/>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" s="11"/>
@@ -2456,11 +2563,12 @@
       <x:c r="K105" s="9"/>
       <x:c r="L105" s="9"/>
       <x:c r="M105" s="10" t="str">
-        <x:f>IF(A105="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O105&lt;&gt;"",O105,IF(A105="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N105" s="10" t="str">
         <x:f>IF(M105="","",LOWER(M105))</x:f>
       </x:c>
+      <x:c r="O105" s="4"/>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" s="11"/>
@@ -2476,11 +2584,12 @@
       <x:c r="K106" s="9"/>
       <x:c r="L106" s="9"/>
       <x:c r="M106" s="10" t="str">
-        <x:f>IF(A106="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O106&lt;&gt;"",O106,IF(A106="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N106" s="10" t="str">
         <x:f>IF(M106="","",LOWER(M106))</x:f>
       </x:c>
+      <x:c r="O106" s="4"/>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" s="11"/>
@@ -2496,11 +2605,12 @@
       <x:c r="K107" s="9"/>
       <x:c r="L107" s="9"/>
       <x:c r="M107" s="10" t="str">
-        <x:f>IF(A107="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000"))</x:f>
+        <x:f>IF(O107&lt;&gt;"",O107,IF(A107="","","HCH-"&amp;$B$3&amp;"-"&amp;TEXT(ROW()-7,"000")))</x:f>
       </x:c>
       <x:c r="N107" s="10" t="str">
         <x:f>IF(M107="","",LOWER(M107))</x:f>
       </x:c>
+      <x:c r="O107" s="4"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="8">
@@ -2601,6 +2711,7 @@
       <x:c r="N1" s="8" t="str">
         <x:v>destacado</x:v>
       </x:c>
+      <x:c r="O1" s="2"/>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="str">
@@ -2645,6 +2756,7 @@
       <x:c r="N2" s="2" t="str">
         <x:f>IF(Productos!L8="","",Productos!L8)</x:f>
       </x:c>
+      <x:c r="O2" s="2"/>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="str">
@@ -2689,6 +2801,7 @@
       <x:c r="N3" s="2" t="str">
         <x:f>IF(Productos!L9="","",Productos!L9)</x:f>
       </x:c>
+      <x:c r="O3" s="2"/>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="str">
@@ -2733,6 +2846,7 @@
       <x:c r="N4" s="2" t="str">
         <x:f>IF(Productos!L10="","",Productos!L10)</x:f>
       </x:c>
+      <x:c r="O4" s="2"/>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="str">
@@ -2777,6 +2891,7 @@
       <x:c r="N5" s="2" t="str">
         <x:f>IF(Productos!L11="","",Productos!L11)</x:f>
       </x:c>
+      <x:c r="O5" s="2"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="str">
@@ -2821,6 +2936,7 @@
       <x:c r="N6" s="2" t="str">
         <x:f>IF(Productos!L12="","",Productos!L12)</x:f>
       </x:c>
+      <x:c r="O6" s="2"/>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="2" t="str">
@@ -2865,6 +2981,7 @@
       <x:c r="N7" s="2" t="str">
         <x:f>IF(Productos!L13="","",Productos!L13)</x:f>
       </x:c>
+      <x:c r="O7" s="2"/>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="2" t="str">
@@ -2909,6 +3026,7 @@
       <x:c r="N8" s="2" t="str">
         <x:f>IF(Productos!L14="","",Productos!L14)</x:f>
       </x:c>
+      <x:c r="O8" s="2"/>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="2" t="str">
@@ -2953,6 +3071,7 @@
       <x:c r="N9" s="2" t="str">
         <x:f>IF(Productos!L15="","",Productos!L15)</x:f>
       </x:c>
+      <x:c r="O9" s="2"/>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="2" t="str">
@@ -2997,6 +3116,7 @@
       <x:c r="N10" s="2" t="str">
         <x:f>IF(Productos!L16="","",Productos!L16)</x:f>
       </x:c>
+      <x:c r="O10" s="2"/>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="2" t="str">
@@ -3041,6 +3161,7 @@
       <x:c r="N11" s="2" t="str">
         <x:f>IF(Productos!L17="","",Productos!L17)</x:f>
       </x:c>
+      <x:c r="O11" s="2"/>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="2" t="str">
@@ -3085,6 +3206,7 @@
       <x:c r="N12" s="2" t="str">
         <x:f>IF(Productos!L18="","",Productos!L18)</x:f>
       </x:c>
+      <x:c r="O12" s="2"/>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="2" t="str">
@@ -3129,6 +3251,7 @@
       <x:c r="N13" s="2" t="str">
         <x:f>IF(Productos!L19="","",Productos!L19)</x:f>
       </x:c>
+      <x:c r="O13" s="2"/>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="2" t="str">
@@ -3173,6 +3296,7 @@
       <x:c r="N14" s="2" t="str">
         <x:f>IF(Productos!L20="","",Productos!L20)</x:f>
       </x:c>
+      <x:c r="O14" s="2"/>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="2" t="str">
@@ -3217,6 +3341,7 @@
       <x:c r="N15" s="2" t="str">
         <x:f>IF(Productos!L21="","",Productos!L21)</x:f>
       </x:c>
+      <x:c r="O15" s="2"/>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="2" t="str">
@@ -3261,6 +3386,7 @@
       <x:c r="N16" s="2" t="str">
         <x:f>IF(Productos!L22="","",Productos!L22)</x:f>
       </x:c>
+      <x:c r="O16" s="2"/>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="2" t="str">
@@ -3305,6 +3431,7 @@
       <x:c r="N17" s="2" t="str">
         <x:f>IF(Productos!L23="","",Productos!L23)</x:f>
       </x:c>
+      <x:c r="O17" s="2"/>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="2" t="str">
@@ -3349,6 +3476,7 @@
       <x:c r="N18" s="2" t="str">
         <x:f>IF(Productos!L24="","",Productos!L24)</x:f>
       </x:c>
+      <x:c r="O18" s="2"/>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="2" t="str">
@@ -3393,6 +3521,7 @@
       <x:c r="N19" s="2" t="str">
         <x:f>IF(Productos!L25="","",Productos!L25)</x:f>
       </x:c>
+      <x:c r="O19" s="2"/>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="2" t="str">
@@ -3437,6 +3566,7 @@
       <x:c r="N20" s="2" t="str">
         <x:f>IF(Productos!L26="","",Productos!L26)</x:f>
       </x:c>
+      <x:c r="O20" s="2"/>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="2" t="str">
@@ -3481,6 +3611,7 @@
       <x:c r="N21" s="2" t="str">
         <x:f>IF(Productos!L27="","",Productos!L27)</x:f>
       </x:c>
+      <x:c r="O21" s="2"/>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="2" t="str">
@@ -3525,6 +3656,7 @@
       <x:c r="N22" s="2" t="str">
         <x:f>IF(Productos!L28="","",Productos!L28)</x:f>
       </x:c>
+      <x:c r="O22" s="2"/>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="2" t="str">
@@ -3569,6 +3701,7 @@
       <x:c r="N23" s="2" t="str">
         <x:f>IF(Productos!L29="","",Productos!L29)</x:f>
       </x:c>
+      <x:c r="O23" s="2"/>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="2" t="str">
@@ -3613,6 +3746,7 @@
       <x:c r="N24" s="2" t="str">
         <x:f>IF(Productos!L30="","",Productos!L30)</x:f>
       </x:c>
+      <x:c r="O24" s="2"/>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="2" t="str">
@@ -3657,6 +3791,7 @@
       <x:c r="N25" s="2" t="str">
         <x:f>IF(Productos!L31="","",Productos!L31)</x:f>
       </x:c>
+      <x:c r="O25" s="2"/>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="2" t="str">
@@ -3701,6 +3836,7 @@
       <x:c r="N26" s="2" t="str">
         <x:f>IF(Productos!L32="","",Productos!L32)</x:f>
       </x:c>
+      <x:c r="O26" s="2"/>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="2" t="str">
@@ -3745,6 +3881,7 @@
       <x:c r="N27" s="2" t="str">
         <x:f>IF(Productos!L33="","",Productos!L33)</x:f>
       </x:c>
+      <x:c r="O27" s="2"/>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="2" t="str">
@@ -3789,6 +3926,7 @@
       <x:c r="N28" s="2" t="str">
         <x:f>IF(Productos!L34="","",Productos!L34)</x:f>
       </x:c>
+      <x:c r="O28" s="2"/>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="2" t="str">
@@ -3833,6 +3971,7 @@
       <x:c r="N29" s="2" t="str">
         <x:f>IF(Productos!L35="","",Productos!L35)</x:f>
       </x:c>
+      <x:c r="O29" s="2"/>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="2" t="str">
@@ -3877,6 +4016,7 @@
       <x:c r="N30" s="2" t="str">
         <x:f>IF(Productos!L36="","",Productos!L36)</x:f>
       </x:c>
+      <x:c r="O30" s="2"/>
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="2" t="str">
@@ -3921,6 +4061,7 @@
       <x:c r="N31" s="2" t="str">
         <x:f>IF(Productos!L37="","",Productos!L37)</x:f>
       </x:c>
+      <x:c r="O31" s="2"/>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="2" t="str">
@@ -3965,6 +4106,7 @@
       <x:c r="N32" s="2" t="str">
         <x:f>IF(Productos!L38="","",Productos!L38)</x:f>
       </x:c>
+      <x:c r="O32" s="2"/>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="2" t="str">
@@ -4009,6 +4151,7 @@
       <x:c r="N33" s="2" t="str">
         <x:f>IF(Productos!L39="","",Productos!L39)</x:f>
       </x:c>
+      <x:c r="O33" s="2"/>
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="2" t="str">
@@ -4053,6 +4196,7 @@
       <x:c r="N34" s="2" t="str">
         <x:f>IF(Productos!L40="","",Productos!L40)</x:f>
       </x:c>
+      <x:c r="O34" s="2"/>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="2" t="str">
@@ -4097,6 +4241,7 @@
       <x:c r="N35" s="2" t="str">
         <x:f>IF(Productos!L41="","",Productos!L41)</x:f>
       </x:c>
+      <x:c r="O35" s="2"/>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="2" t="str">
@@ -4141,6 +4286,7 @@
       <x:c r="N36" s="2" t="str">
         <x:f>IF(Productos!L42="","",Productos!L42)</x:f>
       </x:c>
+      <x:c r="O36" s="2"/>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="2" t="str">
@@ -4185,6 +4331,7 @@
       <x:c r="N37" s="2" t="str">
         <x:f>IF(Productos!L43="","",Productos!L43)</x:f>
       </x:c>
+      <x:c r="O37" s="2"/>
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="2" t="str">
@@ -4229,6 +4376,7 @@
       <x:c r="N38" s="2" t="str">
         <x:f>IF(Productos!L44="","",Productos!L44)</x:f>
       </x:c>
+      <x:c r="O38" s="2"/>
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="2" t="str">
@@ -4273,6 +4421,7 @@
       <x:c r="N39" s="2" t="str">
         <x:f>IF(Productos!L45="","",Productos!L45)</x:f>
       </x:c>
+      <x:c r="O39" s="2"/>
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="2" t="str">
@@ -4317,6 +4466,7 @@
       <x:c r="N40" s="2" t="str">
         <x:f>IF(Productos!L46="","",Productos!L46)</x:f>
       </x:c>
+      <x:c r="O40" s="2"/>
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="2" t="str">
@@ -4361,6 +4511,7 @@
       <x:c r="N41" s="2" t="str">
         <x:f>IF(Productos!L47="","",Productos!L47)</x:f>
       </x:c>
+      <x:c r="O41" s="2"/>
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" s="2" t="str">
@@ -4405,6 +4556,7 @@
       <x:c r="N42" s="2" t="str">
         <x:f>IF(Productos!L48="","",Productos!L48)</x:f>
       </x:c>
+      <x:c r="O42" s="2"/>
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="2" t="str">
@@ -4449,6 +4601,7 @@
       <x:c r="N43" s="2" t="str">
         <x:f>IF(Productos!L49="","",Productos!L49)</x:f>
       </x:c>
+      <x:c r="O43" s="2"/>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="2" t="str">
@@ -4493,6 +4646,7 @@
       <x:c r="N44" s="2" t="str">
         <x:f>IF(Productos!L50="","",Productos!L50)</x:f>
       </x:c>
+      <x:c r="O44" s="2"/>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" s="2" t="str">
@@ -4537,6 +4691,7 @@
       <x:c r="N45" s="2" t="str">
         <x:f>IF(Productos!L51="","",Productos!L51)</x:f>
       </x:c>
+      <x:c r="O45" s="2"/>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" s="2" t="str">
@@ -4581,6 +4736,7 @@
       <x:c r="N46" s="2" t="str">
         <x:f>IF(Productos!L52="","",Productos!L52)</x:f>
       </x:c>
+      <x:c r="O46" s="2"/>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" s="2" t="str">
@@ -4625,6 +4781,7 @@
       <x:c r="N47" s="2" t="str">
         <x:f>IF(Productos!L53="","",Productos!L53)</x:f>
       </x:c>
+      <x:c r="O47" s="2"/>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" s="2" t="str">
@@ -4669,6 +4826,7 @@
       <x:c r="N48" s="2" t="str">
         <x:f>IF(Productos!L54="","",Productos!L54)</x:f>
       </x:c>
+      <x:c r="O48" s="2"/>
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" s="2" t="str">
@@ -4713,6 +4871,7 @@
       <x:c r="N49" s="2" t="str">
         <x:f>IF(Productos!L55="","",Productos!L55)</x:f>
       </x:c>
+      <x:c r="O49" s="2"/>
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" s="2" t="str">
@@ -4757,6 +4916,7 @@
       <x:c r="N50" s="2" t="str">
         <x:f>IF(Productos!L56="","",Productos!L56)</x:f>
       </x:c>
+      <x:c r="O50" s="2"/>
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" s="2" t="str">
@@ -4801,6 +4961,7 @@
       <x:c r="N51" s="2" t="str">
         <x:f>IF(Productos!L57="","",Productos!L57)</x:f>
       </x:c>
+      <x:c r="O51" s="2"/>
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" s="2" t="str">
@@ -4845,6 +5006,7 @@
       <x:c r="N52" s="2" t="str">
         <x:f>IF(Productos!L58="","",Productos!L58)</x:f>
       </x:c>
+      <x:c r="O52" s="2"/>
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" s="2" t="str">
@@ -4889,6 +5051,7 @@
       <x:c r="N53" s="2" t="str">
         <x:f>IF(Productos!L59="","",Productos!L59)</x:f>
       </x:c>
+      <x:c r="O53" s="2"/>
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" s="2" t="str">
@@ -4933,6 +5096,7 @@
       <x:c r="N54" s="2" t="str">
         <x:f>IF(Productos!L60="","",Productos!L60)</x:f>
       </x:c>
+      <x:c r="O54" s="2"/>
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" s="2" t="str">
@@ -4977,6 +5141,7 @@
       <x:c r="N55" s="2" t="str">
         <x:f>IF(Productos!L61="","",Productos!L61)</x:f>
       </x:c>
+      <x:c r="O55" s="2"/>
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" s="2" t="str">
@@ -5021,6 +5186,7 @@
       <x:c r="N56" s="2" t="str">
         <x:f>IF(Productos!L62="","",Productos!L62)</x:f>
       </x:c>
+      <x:c r="O56" s="2"/>
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" s="2" t="str">
@@ -5065,6 +5231,7 @@
       <x:c r="N57" s="2" t="str">
         <x:f>IF(Productos!L63="","",Productos!L63)</x:f>
       </x:c>
+      <x:c r="O57" s="2"/>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" s="2" t="str">
@@ -5109,6 +5276,7 @@
       <x:c r="N58" s="2" t="str">
         <x:f>IF(Productos!L64="","",Productos!L64)</x:f>
       </x:c>
+      <x:c r="O58" s="2"/>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" s="2" t="str">
@@ -5153,6 +5321,7 @@
       <x:c r="N59" s="2" t="str">
         <x:f>IF(Productos!L65="","",Productos!L65)</x:f>
       </x:c>
+      <x:c r="O59" s="2"/>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" s="2" t="str">
@@ -5197,6 +5366,7 @@
       <x:c r="N60" s="2" t="str">
         <x:f>IF(Productos!L66="","",Productos!L66)</x:f>
       </x:c>
+      <x:c r="O60" s="2"/>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" s="2" t="str">
@@ -5241,6 +5411,7 @@
       <x:c r="N61" s="2" t="str">
         <x:f>IF(Productos!L67="","",Productos!L67)</x:f>
       </x:c>
+      <x:c r="O61" s="2"/>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" s="2" t="str">
@@ -5285,6 +5456,7 @@
       <x:c r="N62" s="2" t="str">
         <x:f>IF(Productos!L68="","",Productos!L68)</x:f>
       </x:c>
+      <x:c r="O62" s="2"/>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" s="2" t="str">
@@ -5329,6 +5501,7 @@
       <x:c r="N63" s="2" t="str">
         <x:f>IF(Productos!L69="","",Productos!L69)</x:f>
       </x:c>
+      <x:c r="O63" s="2"/>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" s="2" t="str">
@@ -5373,6 +5546,7 @@
       <x:c r="N64" s="2" t="str">
         <x:f>IF(Productos!L70="","",Productos!L70)</x:f>
       </x:c>
+      <x:c r="O64" s="2"/>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" s="2" t="str">
@@ -5417,6 +5591,7 @@
       <x:c r="N65" s="2" t="str">
         <x:f>IF(Productos!L71="","",Productos!L71)</x:f>
       </x:c>
+      <x:c r="O65" s="2"/>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" s="2" t="str">
@@ -5461,6 +5636,7 @@
       <x:c r="N66" s="2" t="str">
         <x:f>IF(Productos!L72="","",Productos!L72)</x:f>
       </x:c>
+      <x:c r="O66" s="2"/>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" s="2" t="str">
@@ -5505,6 +5681,7 @@
       <x:c r="N67" s="2" t="str">
         <x:f>IF(Productos!L73="","",Productos!L73)</x:f>
       </x:c>
+      <x:c r="O67" s="2"/>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" s="2" t="str">
@@ -5549,6 +5726,7 @@
       <x:c r="N68" s="2" t="str">
         <x:f>IF(Productos!L74="","",Productos!L74)</x:f>
       </x:c>
+      <x:c r="O68" s="2"/>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" s="2" t="str">
@@ -5593,6 +5771,7 @@
       <x:c r="N69" s="2" t="str">
         <x:f>IF(Productos!L75="","",Productos!L75)</x:f>
       </x:c>
+      <x:c r="O69" s="2"/>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" s="2" t="str">
@@ -5637,6 +5816,7 @@
       <x:c r="N70" s="2" t="str">
         <x:f>IF(Productos!L76="","",Productos!L76)</x:f>
       </x:c>
+      <x:c r="O70" s="2"/>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" s="2" t="str">
@@ -5681,6 +5861,7 @@
       <x:c r="N71" s="2" t="str">
         <x:f>IF(Productos!L77="","",Productos!L77)</x:f>
       </x:c>
+      <x:c r="O71" s="2"/>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" s="2" t="str">
@@ -5725,6 +5906,7 @@
       <x:c r="N72" s="2" t="str">
         <x:f>IF(Productos!L78="","",Productos!L78)</x:f>
       </x:c>
+      <x:c r="O72" s="2"/>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" s="2" t="str">
@@ -5769,6 +5951,7 @@
       <x:c r="N73" s="2" t="str">
         <x:f>IF(Productos!L79="","",Productos!L79)</x:f>
       </x:c>
+      <x:c r="O73" s="2"/>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" s="2" t="str">
@@ -5813,6 +5996,7 @@
       <x:c r="N74" s="2" t="str">
         <x:f>IF(Productos!L80="","",Productos!L80)</x:f>
       </x:c>
+      <x:c r="O74" s="2"/>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" s="2" t="str">
@@ -5857,6 +6041,7 @@
       <x:c r="N75" s="2" t="str">
         <x:f>IF(Productos!L81="","",Productos!L81)</x:f>
       </x:c>
+      <x:c r="O75" s="2"/>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" s="2" t="str">
@@ -5901,6 +6086,7 @@
       <x:c r="N76" s="2" t="str">
         <x:f>IF(Productos!L82="","",Productos!L82)</x:f>
       </x:c>
+      <x:c r="O76" s="2"/>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" s="2" t="str">
@@ -5945,6 +6131,7 @@
       <x:c r="N77" s="2" t="str">
         <x:f>IF(Productos!L83="","",Productos!L83)</x:f>
       </x:c>
+      <x:c r="O77" s="2"/>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" s="2" t="str">
@@ -5989,6 +6176,7 @@
       <x:c r="N78" s="2" t="str">
         <x:f>IF(Productos!L84="","",Productos!L84)</x:f>
       </x:c>
+      <x:c r="O78" s="2"/>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" s="2" t="str">
@@ -6033,6 +6221,7 @@
       <x:c r="N79" s="2" t="str">
         <x:f>IF(Productos!L85="","",Productos!L85)</x:f>
       </x:c>
+      <x:c r="O79" s="2"/>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" s="2" t="str">
@@ -6077,6 +6266,7 @@
       <x:c r="N80" s="2" t="str">
         <x:f>IF(Productos!L86="","",Productos!L86)</x:f>
       </x:c>
+      <x:c r="O80" s="2"/>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" s="2" t="str">
@@ -6121,6 +6311,7 @@
       <x:c r="N81" s="2" t="str">
         <x:f>IF(Productos!L87="","",Productos!L87)</x:f>
       </x:c>
+      <x:c r="O81" s="2"/>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" s="2" t="str">
@@ -6165,6 +6356,7 @@
       <x:c r="N82" s="2" t="str">
         <x:f>IF(Productos!L88="","",Productos!L88)</x:f>
       </x:c>
+      <x:c r="O82" s="2"/>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" s="2" t="str">
@@ -6209,6 +6401,7 @@
       <x:c r="N83" s="2" t="str">
         <x:f>IF(Productos!L89="","",Productos!L89)</x:f>
       </x:c>
+      <x:c r="O83" s="2"/>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" s="2" t="str">
@@ -6253,6 +6446,7 @@
       <x:c r="N84" s="2" t="str">
         <x:f>IF(Productos!L90="","",Productos!L90)</x:f>
       </x:c>
+      <x:c r="O84" s="2"/>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" s="2" t="str">
@@ -6297,6 +6491,7 @@
       <x:c r="N85" s="2" t="str">
         <x:f>IF(Productos!L91="","",Productos!L91)</x:f>
       </x:c>
+      <x:c r="O85" s="2"/>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" s="2" t="str">
@@ -6341,6 +6536,7 @@
       <x:c r="N86" s="2" t="str">
         <x:f>IF(Productos!L92="","",Productos!L92)</x:f>
       </x:c>
+      <x:c r="O86" s="2"/>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" s="2" t="str">
@@ -6385,6 +6581,7 @@
       <x:c r="N87" s="2" t="str">
         <x:f>IF(Productos!L93="","",Productos!L93)</x:f>
       </x:c>
+      <x:c r="O87" s="2"/>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" s="2" t="str">
@@ -6429,6 +6626,7 @@
       <x:c r="N88" s="2" t="str">
         <x:f>IF(Productos!L94="","",Productos!L94)</x:f>
       </x:c>
+      <x:c r="O88" s="2"/>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" s="2" t="str">
@@ -6473,6 +6671,7 @@
       <x:c r="N89" s="2" t="str">
         <x:f>IF(Productos!L95="","",Productos!L95)</x:f>
       </x:c>
+      <x:c r="O89" s="2"/>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" s="2" t="str">
@@ -6517,6 +6716,7 @@
       <x:c r="N90" s="2" t="str">
         <x:f>IF(Productos!L96="","",Productos!L96)</x:f>
       </x:c>
+      <x:c r="O90" s="2"/>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" s="2" t="str">
@@ -6561,6 +6761,7 @@
       <x:c r="N91" s="2" t="str">
         <x:f>IF(Productos!L97="","",Productos!L97)</x:f>
       </x:c>
+      <x:c r="O91" s="2"/>
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" s="2" t="str">
@@ -6605,6 +6806,7 @@
       <x:c r="N92" s="2" t="str">
         <x:f>IF(Productos!L98="","",Productos!L98)</x:f>
       </x:c>
+      <x:c r="O92" s="2"/>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" s="2" t="str">
@@ -6649,6 +6851,7 @@
       <x:c r="N93" s="2" t="str">
         <x:f>IF(Productos!L99="","",Productos!L99)</x:f>
       </x:c>
+      <x:c r="O93" s="2"/>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" s="2" t="str">
@@ -6693,6 +6896,7 @@
       <x:c r="N94" s="2" t="str">
         <x:f>IF(Productos!L100="","",Productos!L100)</x:f>
       </x:c>
+      <x:c r="O94" s="2"/>
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" s="2" t="str">
@@ -6737,6 +6941,7 @@
       <x:c r="N95" s="2" t="str">
         <x:f>IF(Productos!L101="","",Productos!L101)</x:f>
       </x:c>
+      <x:c r="O95" s="2"/>
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" s="2" t="str">
@@ -6781,6 +6986,7 @@
       <x:c r="N96" s="2" t="str">
         <x:f>IF(Productos!L102="","",Productos!L102)</x:f>
       </x:c>
+      <x:c r="O96" s="2"/>
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" s="2" t="str">
@@ -6825,6 +7031,7 @@
       <x:c r="N97" s="2" t="str">
         <x:f>IF(Productos!L103="","",Productos!L103)</x:f>
       </x:c>
+      <x:c r="O97" s="2"/>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" s="2" t="str">
@@ -6869,6 +7076,7 @@
       <x:c r="N98" s="2" t="str">
         <x:f>IF(Productos!L104="","",Productos!L104)</x:f>
       </x:c>
+      <x:c r="O98" s="2"/>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" s="2" t="str">
@@ -6913,6 +7121,7 @@
       <x:c r="N99" s="2" t="str">
         <x:f>IF(Productos!L105="","",Productos!L105)</x:f>
       </x:c>
+      <x:c r="O99" s="2"/>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" s="2" t="str">
@@ -6957,6 +7166,7 @@
       <x:c r="N100" s="2" t="str">
         <x:f>IF(Productos!L106="","",Productos!L106)</x:f>
       </x:c>
+      <x:c r="O100" s="2"/>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" s="2" t="str">
@@ -7001,6 +7211,7 @@
       <x:c r="N101" s="2" t="str">
         <x:f>IF(Productos!L107="","",Productos!L107)</x:f>
       </x:c>
+      <x:c r="O101" s="2"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="2"/>
@@ -7017,6 +7228,7 @@
       <x:c r="L102" s="2"/>
       <x:c r="M102" s="2"/>
       <x:c r="N102" s="2"/>
+      <x:c r="O102" s="2"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="2"/>
@@ -7033,6 +7245,7 @@
       <x:c r="L103" s="2"/>
       <x:c r="M103" s="2"/>
       <x:c r="N103" s="2"/>
+      <x:c r="O103" s="2"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="2"/>
@@ -7049,6 +7262,7 @@
       <x:c r="L104" s="2"/>
       <x:c r="M104" s="2"/>
       <x:c r="N104" s="2"/>
+      <x:c r="O104" s="2"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="2"/>
@@ -7065,6 +7279,7 @@
       <x:c r="L105" s="2"/>
       <x:c r="M105" s="2"/>
       <x:c r="N105" s="2"/>
+      <x:c r="O105" s="2"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="2"/>
@@ -7081,6 +7296,7 @@
       <x:c r="L106" s="2"/>
       <x:c r="M106" s="2"/>
       <x:c r="N106" s="2"/>
+      <x:c r="O106" s="2"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="2"/>
@@ -7097,6 +7313,7 @@
       <x:c r="L107" s="2"/>
       <x:c r="M107" s="2"/>
       <x:c r="N107" s="2"/>
+      <x:c r="O107" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7136,7 +7353,7 @@
         <x:v>Paso 1</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>Edita Productos. Amarillo = editable; gris = fórmula automática. Hay 100 filas preparadas.</x:v>
+        <x:v>Producto nuevo: completa Nombre, Descripción, Categoría, Precio, Stock y Peso en una fila.</x:v>
       </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
@@ -7146,7 +7363,7 @@
         <x:v>Paso 2</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>Elige categoría en el desplegable. Los campos con * son obligatorios. Precios en pesos enteros.</x:v>
+        <x:v>Reposición: escribe solo el SKU existente en la columna O y la cantidad a sumar en Stock (columna E).</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2"/>
@@ -7156,7 +7373,7 @@
         <x:v>Paso 3</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>Al escribir el nombre aparece el SKU. La URL se calcula desde ese SKU; no necesitas escribirlos.</x:v>
+        <x:v>Amarillo = editable; gris = fórmula. Para productos nuevos, SKU y URL se calculan automáticamente.</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2"/>
@@ -7196,7 +7413,7 @@
         <x:v>Evita duplicados</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>El código de lote + número de fila forman el SKU. Conserva el mismo código al reintentar una importación.</x:v>
+        <x:v>El código de lote + fila forman el SKU nuevo. Reimportar una reposición sumará el stock otra vez.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -7263,10 +7480,10 @@
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:v>Stock (un.)</x:v>
+        <x:v>Stock / sumar</x:v>
       </x:c>
       <x:c r="B17" s="13" t="str">
-        <x:v>Cantidad inicial disponible: entero desde 0. La importación registra el movimiento de inventario.</x:v>
+        <x:v>Producto nuevo: stock inicial desde 0. SKU existente: cantidad positiva a sumar al stock actual.</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="2"/>
@@ -7336,7 +7553,7 @@
         <x:v>SKU / URL</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>Identificadores únicos. Si ya existen, se rechaza el archivo completo; esta carga no actualiza productos.</x:v>
+        <x:v>El SKU identifica un producto sin variantes. Un SKU existente solo suma stock; no cambia los demás datos.</x:v>
       </x:c>
       <x:c r="C24" s="2"/>
       <x:c r="D24" s="2"/>
@@ -7356,7 +7573,7 @@
         <x:v>Plantilla vacía</x:v>
       </x:c>
       <x:c r="B26" s="13" t="str">
-        <x:v>No hay productos cargados en este archivo. Completa Nombre, Descripción, Categoría, Precio, Stock y Peso.</x:v>
+        <x:v>No hay productos cargados. Puedes combinar filas nuevas y reposiciones en el mismo archivo.</x:v>
       </x:c>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="2"/>

</xml_diff>